<commit_message>
Version completamente funcional sin correo
</commit_message>
<xml_diff>
--- a/Plantilla_export_pedidos.xlsx
+++ b/Plantilla_export_pedidos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/jhor_caro_quotamedia_co/Documents/Documentos/GitHub/App_Pedidos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="121" documentId="11_AD4D2F04E46CFB4ACB3E20F1CD94FB2A693EDF13" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EBA8AF9F-92E2-4527-A064-EAF4C811DF40}"/>
+  <xr:revisionPtr revIDLastSave="126" documentId="11_AD4D2F04E46CFB4ACB3E20F1CD94FB2A693EDF13" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9F66E2E-BAAC-4631-B580-0404ED94BB0E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -118,7 +118,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="44" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="_-&quot;$&quot;\ * #,##0_-;\-&quot;$&quot;\ * #,##0_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -136,6 +140,13 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -313,10 +324,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -335,6 +347,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -344,9 +359,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -371,8 +383,12 @@
     <xf numFmtId="14" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="166" fontId="2" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="4" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Moneda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -664,27 +680,27 @@
     <col min="8" max="8" width="11" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.5703125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="27.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
-      <c r="K1" s="13"/>
-      <c r="L1" s="13"/>
-      <c r="M1" s="14"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
+      <c r="L1" s="14"/>
+      <c r="M1" s="15"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
@@ -734,22 +750,22 @@
       <c r="B3" s="23">
         <v>46142</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="15" t="s">
+      <c r="G3" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="15">
+      <c r="H3" s="12">
         <v>3017333166</v>
       </c>
       <c r="I3" s="4" t="s">
@@ -758,10 +774,10 @@
       <c r="J3" s="4">
         <v>10</v>
       </c>
-      <c r="K3" s="4">
+      <c r="K3" s="24">
         <v>13500</v>
       </c>
-      <c r="L3" s="4">
+      <c r="L3" s="24">
         <v>135000</v>
       </c>
       <c r="M3" s="6" t="s">
@@ -771,22 +787,22 @@
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="22"/>
       <c r="B4" s="23"/>
-      <c r="C4" s="15"/>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
-      <c r="H4" s="15"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
       <c r="I4" s="4" t="s">
         <v>20</v>
       </c>
       <c r="J4" s="4">
         <v>10</v>
       </c>
-      <c r="K4" s="4">
+      <c r="K4" s="24">
         <v>6500</v>
       </c>
-      <c r="L4" s="4">
+      <c r="L4" s="24">
         <v>65000</v>
       </c>
       <c r="M4" s="6"/>
@@ -794,22 +810,22 @@
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="22"/>
       <c r="B5" s="23"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="12"/>
       <c r="I5" s="4" t="s">
         <v>21</v>
       </c>
       <c r="J5" s="4">
         <v>20</v>
       </c>
-      <c r="K5" s="4">
+      <c r="K5" s="24">
         <v>4000</v>
       </c>
-      <c r="L5" s="4">
+      <c r="L5" s="24">
         <v>80000</v>
       </c>
       <c r="M5" s="6"/>
@@ -845,10 +861,10 @@
       <c r="J6" s="5">
         <v>10</v>
       </c>
-      <c r="K6" s="5">
+      <c r="K6" s="25">
         <v>4000</v>
       </c>
-      <c r="L6" s="5">
+      <c r="L6" s="25">
         <v>40000</v>
       </c>
       <c r="M6" s="7"/>
@@ -868,10 +884,10 @@
       <c r="J7" s="8">
         <v>100</v>
       </c>
-      <c r="K7" s="8">
+      <c r="K7" s="26">
         <v>14000</v>
       </c>
-      <c r="L7" s="8">
+      <c r="L7" s="26">
         <v>1400000</v>
       </c>
       <c r="M7" s="9" t="s">
@@ -880,6 +896,7 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="E3:E5"/>
     <mergeCell ref="F3:F5"/>
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="G3:G5"/>
@@ -896,7 +913,6 @@
     <mergeCell ref="B3:B5"/>
     <mergeCell ref="C3:C5"/>
     <mergeCell ref="D3:D5"/>
-    <mergeCell ref="E3:E5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>